<commit_message>
Correcciones en generación de reporte
</commit_message>
<xml_diff>
--- a/src/test/resources/data/TestData.xlsx
+++ b/src/test/resources/data/TestData.xlsx
@@ -4,20 +4,21 @@
   <workbookPr/>
   <sheets>
     <sheet state="visible" name="Login" sheetId="1" r:id="rId4"/>
-    <sheet state="visible" name="CambioDeDispositivo" sheetId="2" r:id="rId5"/>
+    <sheet state="visible" name="CambioDispositivo" sheetId="2" r:id="rId5"/>
+    <sheet state="visible" name="CambioClave" sheetId="3" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="LI4udGZVDaDKMJgksJm/6vvIS2ph2uY5mgtAx3HmR2c="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId7" roundtripDataChecksum="yER+5tvrRrDuCRclhdqAaAsjnA/71gyUz9jDTYnobP4="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="38">
   <si>
     <t>tipoId</t>
   </si>
@@ -58,7 +59,7 @@
     <t>@CP0003</t>
   </si>
   <si>
-    <t>DAVIPLATA</t>
+    <t>DAV</t>
   </si>
   <si>
     <t>@CP0004</t>
@@ -88,6 +89,9 @@
     <t>@CP0011</t>
   </si>
   <si>
+    <t>RAP</t>
+  </si>
+  <si>
     <t>@CP0012</t>
   </si>
   <si>
@@ -95,6 +99,39 @@
   </si>
   <si>
     <t>@CP0014</t>
+  </si>
+  <si>
+    <t>newPass</t>
+  </si>
+  <si>
+    <t>subTipo</t>
+  </si>
+  <si>
+    <t>@CP0015</t>
+  </si>
+  <si>
+    <t>@CP0016</t>
+  </si>
+  <si>
+    <t>@CP0017</t>
+  </si>
+  <si>
+    <t>@CP0018</t>
+  </si>
+  <si>
+    <t>@CP0019</t>
+  </si>
+  <si>
+    <t>@CP0020</t>
+  </si>
+  <si>
+    <t>@CP0021</t>
+  </si>
+  <si>
+    <t>@CP0022</t>
+  </si>
+  <si>
+    <t>@CP0023</t>
   </si>
 </sst>
 </file>
@@ -189,6 +226,10 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -440,13 +481,13 @@
         <v>999837.0</v>
       </c>
       <c r="C2" s="3">
-        <v>1234.0</v>
+        <v>1111.0</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>7</v>
       </c>
       <c r="E2" s="3">
-        <v>3.142045585E9</v>
+        <v>3.142045565E9</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>8</v>
@@ -561,11 +602,11 @@
       <c r="A6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="5">
-        <v>578711.0</v>
+      <c r="B6" s="3">
+        <v>999842.0</v>
       </c>
       <c r="C6" s="3">
-        <v>2580.0</v>
+        <v>1111.0</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>15</v>
@@ -578,23 +619,19 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" s="5">
-        <v>578711.0</v>
+      <c r="A7" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="3">
+        <v>999829.0</v>
       </c>
       <c r="C7" s="3">
-        <v>2580.0</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E7" s="3">
-        <v>3.142045595E9</v>
-      </c>
+        <v>2589.0</v>
+      </c>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
       <c r="F7" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8">
@@ -610,30 +647,14 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" s="3">
-        <v>999829.0</v>
-      </c>
-      <c r="C9" s="3">
-        <v>2589.0</v>
-      </c>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3" t="s">
-        <v>18</v>
-      </c>
+      <c r="H9" s="6"/>
     </row>
     <row r="10">
       <c r="H10" s="6"/>
-    </row>
-    <row r="11">
-      <c r="H11" s="6"/>
     </row>
   </sheetData>
   <printOptions/>
@@ -649,9 +670,6 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
-  <cols>
-    <col customWidth="1" min="5" max="5" width="18.0"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -667,7 +685,153 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="3">
+        <v>999837.0</v>
+      </c>
+      <c r="C2" s="3">
+        <v>1111.0</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="3">
+        <v>999829.0</v>
+      </c>
+      <c r="C3" s="3">
+        <v>2580.0</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="3">
+        <v>1.080406492E9</v>
+      </c>
+      <c r="C4" s="3">
+        <v>1234.0</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="3">
+        <v>999906.0</v>
+      </c>
+      <c r="C5" s="3">
+        <v>1234.0</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="3">
+        <v>9999815.0</v>
+      </c>
+      <c r="C6" s="3">
+        <v>1234.0</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3">
+        <v>999842.0</v>
+      </c>
+      <c r="C7" s="3">
+        <v>1111.0</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3">
+        <v>9999815.0</v>
+      </c>
+      <c r="C8" s="3">
+        <v>2589.0</v>
+      </c>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>28</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>5</v>
@@ -678,59 +842,59 @@
         <v>6</v>
       </c>
       <c r="B2" s="3">
-        <v>999837.0</v>
+        <v>666710.0</v>
       </c>
       <c r="C2" s="3">
-        <v>1234.0</v>
-      </c>
-      <c r="D2" s="3" t="s">
+        <v>1113.0</v>
+      </c>
+      <c r="D2" s="3">
+        <v>1114.0</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="3">
-        <v>3.142045585E9</v>
-      </c>
       <c r="F2" s="3" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="3">
+        <v>666711.0</v>
+      </c>
+      <c r="C3" s="3">
+        <v>1113.0</v>
+      </c>
+      <c r="D3" s="3">
+        <v>1114.0</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="3">
-        <v>1.080406492E9</v>
-      </c>
-      <c r="C3" s="3">
-        <v>1234.0</v>
-      </c>
-      <c r="D3" s="3" t="s">
+      <c r="B4" s="3">
+        <v>666712.0</v>
+      </c>
+      <c r="C4" s="3">
+        <v>1114.0</v>
+      </c>
+      <c r="D4" s="3">
+        <v>1115.0</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="3">
-        <v>3.142045552E9</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="3">
-        <v>999829.0</v>
-      </c>
-      <c r="C4" s="3">
-        <v>2580.0</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" s="3">
-        <v>3.142204551E9</v>
-      </c>
       <c r="F4" s="3" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5">
@@ -738,91 +902,113 @@
         <v>6</v>
       </c>
       <c r="B5" s="3">
-        <v>999798.0</v>
+        <v>999730.0</v>
       </c>
       <c r="C5" s="3">
-        <v>1111.0</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" s="3">
-        <v>3.004005051E9</v>
+        <v>1112.0</v>
+      </c>
+      <c r="D5" s="3">
+        <v>1113.0</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="5">
-        <v>578711.0</v>
+      <c r="B6" s="3">
+        <v>999840.0</v>
       </c>
       <c r="C6" s="3">
-        <v>2580.0</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" s="3">
-        <v>3.142045595E9</v>
+        <v>1111.0</v>
+      </c>
+      <c r="D6" s="3">
+        <v>1112.0</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>23</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="5">
-        <v>578711.0</v>
+      <c r="B7" s="3">
+        <v>4.621523583E9</v>
       </c>
       <c r="C7" s="3">
-        <v>2580.0</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E7" s="3">
-        <v>3.142045595E9</v>
+        <v>1111.0</v>
+      </c>
+      <c r="D7" s="3">
+        <v>1112.0</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>7</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="B8" s="3">
-        <v>999829.0</v>
+        <v>999901.0</v>
       </c>
       <c r="C8" s="3">
-        <v>2589.0</v>
-      </c>
-      <c r="D8" s="3"/>
+        <v>1111.0</v>
+      </c>
+      <c r="D8" s="3">
+        <v>1900.0</v>
+      </c>
       <c r="E8" s="3"/>
       <c r="F8" s="3" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="B9" s="3">
-        <v>999829.0</v>
+        <v>999901.0</v>
       </c>
       <c r="C9" s="3">
-        <v>2589.0</v>
-      </c>
-      <c r="D9" s="3"/>
+        <v>1111.0</v>
+      </c>
+      <c r="D9" s="3">
+        <v>1111.0</v>
+      </c>
       <c r="E9" s="3"/>
       <c r="F9" s="3" t="s">
-        <v>25</v>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="3">
+        <v>2.0331723E7</v>
+      </c>
+      <c r="C10" s="3">
+        <v>1112.0</v>
+      </c>
+      <c r="D10" s="3">
+        <v>1113.0</v>
+      </c>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>